<commit_message>
Update IŞIK PETROL analysis - group by date ranges
- Changed grouping from row numbers to date ranges
- 01.06.2026 - 10.06.2026: 21 işlem, 1130.07 TL
- 11.06.2026 - 20.06.2026: 20 işlem, 1493.42 TL
- 21.06.2026 - 30.06.2026: 15 işlem, 837.48 TL
- Genel Toplam: 56 işlem, 3460.97 TL
</commit_message>
<xml_diff>
--- a/ISIK_PETROL_GARANT_OZET.xlsx
+++ b/ISIK_PETROL_GARANT_OZET.xlsx
@@ -28,12 +28,14 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
         <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,15 +73,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,18 +456,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Satır Aralığı</t>
+          <t>Tarih Aralığı</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -467,53 +484,53 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>01.06.2026 - 10.06.2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>162.06</v>
+        <v>1130.07</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>11-20</t>
+          <t>11.06.2026 - 20.06.2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>447.67</v>
+        <v>1493.42</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>21-30</t>
+          <t>21.06.2026 - 30.06.2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>182.28</v>
+        <v>837.4799999999999</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>792.01</v>
+      <c r="B6" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>3460.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>